<commit_message>
Final update for June 4
</commit_message>
<xml_diff>
--- a/AutoReadUSBRData/Bathymetry.xlsx
+++ b/AutoReadUSBRData/Bathymetry.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Rosenberg\Work\USU\Research\ColoradoRiver\RCode\ColoradoRiverCollaborate\AutoReadUSBRData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F6EEA5B-4BE3-4F98-8A31-75CA1533DB92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{243191D9-FC4E-4B5F-A2BD-07236EC240D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-23280" yWindow="675" windowWidth="21600" windowHeight="11175" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ReadMe" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="27">
   <si>
     <t>Elevation (ft)</t>
   </si>
@@ -115,6 +115,27 @@
   <si>
     <t>Taken from Bradley, D., and Collins, K. (2022). "Lake Powell 2017 Area and Capacity Tables." ENV-2021-98, Reclamation. https://doi.org/10.5066/P9O3IPG3. See also folder LakePowellNewBathymetry</t>
   </si>
+  <si>
+    <t>Reservoir</t>
+  </si>
+  <si>
+    <t>Lake Powell</t>
+  </si>
+  <si>
+    <t>Lake Mead</t>
+  </si>
+  <si>
+    <t>Elevation (feet)</t>
+  </si>
+  <si>
+    <t>Total Storage (maf)</t>
+  </si>
+  <si>
+    <t>Active Storage (maf)</t>
+  </si>
+  <si>
+    <t>Calculator. Enter Elevation (peach fill) and spreadsheet will calculate Total Storage and Active Storage (grey fill).</t>
+  </si>
 </sst>
 </file>
 
@@ -126,7 +147,7 @@
     <numFmt numFmtId="165" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="166" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -190,8 +211,23 @@
       <name val="Times New Roman"/>
       <family val="1"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -204,8 +240,24 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="3">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -231,14 +283,46 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="4">
+  <cellStyleXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="3" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="3" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -326,10 +410,23 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="3" xfId="4" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="11" fillId="4" borderId="3" xfId="5" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="4">
+  <cellStyles count="6">
+    <cellStyle name="Calculation" xfId="5" builtinId="22"/>
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
     <cellStyle name="Comma 2" xfId="3" xr:uid="{4202C67F-73A5-4984-9593-8DDD62E3EDD3}"/>
+    <cellStyle name="Input" xfId="4" builtinId="20"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="2" xr:uid="{61877EEE-4DD3-4165-A074-4E8B8BC7255E}"/>
   </cellStyles>
@@ -9253,23 +9350,25 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:D13"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="16.36328125" customWidth="1"/>
+    <col min="3" max="3" width="9.54296875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>12</v>
       </c>
@@ -9277,7 +9376,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>14</v>
       </c>
@@ -9285,12 +9384,63 @@
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>16</v>
       </c>
       <c r="B6" t="s">
         <v>19</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A9" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A11" s="33" t="s">
+        <v>20</v>
+      </c>
+      <c r="B11" s="34" t="s">
+        <v>23</v>
+      </c>
+      <c r="C11" s="34" t="s">
+        <v>24</v>
+      </c>
+      <c r="D11" s="34" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A12" s="35" t="s">
+        <v>21</v>
+      </c>
+      <c r="B12" s="36">
+        <v>3510</v>
+      </c>
+      <c r="C12" s="37">
+        <f>VLOOKUP(B12,'Powell-Bathymetry'!$B$2:$C$582,2)/1000000</f>
+        <v>6.433061801</v>
+      </c>
+      <c r="D12" s="37">
+        <f>C12-VLOOKUP(3370,'Powell-Bathymetry'!$B$2:$C$582,2)/1000000</f>
+        <v>4.7210644459999997</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A13" s="35" t="s">
+        <v>22</v>
+      </c>
+      <c r="B13" s="36">
+        <v>1000</v>
+      </c>
+      <c r="C13" s="37">
+        <f>VLOOKUP(B$13,'Mead-Bathymetry'!$A$2:$D$673,3)/1000000</f>
+        <v>6.5103010000000001</v>
+      </c>
+      <c r="D13" s="37">
+        <f>VLOOKUP(B$13,'Mead-Bathymetry'!$A$2:$D$673,2)/1000000</f>
+        <v>4.475301</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Tweaking sub Powell plot to show buffer volume
</commit_message>
<xml_diff>
--- a/AutoReadUSBRData/Bathymetry.xlsx
+++ b/AutoReadUSBRData/Bathymetry.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Rosenberg\Work\USU\Research\ColoradoRiver\RCode\ColoradoRiverCollaborate\AutoReadUSBRData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{243191D9-FC4E-4B5F-A2BD-07236EC240D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{986D7C98-EC2A-413C-BD64-6CFBD01ADE7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-23280" yWindow="675" windowWidth="21600" windowHeight="11175" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-57720" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ReadMe" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="29">
   <si>
     <t>Elevation (ft)</t>
   </si>
@@ -135,6 +135,12 @@
   </si>
   <si>
     <t>Calculator. Enter Elevation (peach fill) and spreadsheet will calculate Total Storage and Active Storage (grey fill).</t>
+  </si>
+  <si>
+    <t>Powell elevation</t>
+  </si>
+  <si>
+    <t>Volume above 3,514</t>
   </si>
 </sst>
 </file>
@@ -322,7 +328,7 @@
     <xf numFmtId="0" fontId="10" fillId="3" borderId="3" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="11" fillId="4" borderId="3" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -420,6 +426,10 @@
     </xf>
     <xf numFmtId="2" fontId="11" fillId="4" borderId="3" xfId="5" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -9350,7 +9360,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:K19"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="16.36328125" customWidth="1"/>
@@ -9358,17 +9368,17 @@
     <col min="4" max="4" width="11.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>12</v>
       </c>
@@ -9376,7 +9386,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>14</v>
       </c>
@@ -9384,7 +9394,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>16</v>
       </c>
@@ -9392,12 +9402,12 @@
         <v>19</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:4" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A11" s="33" t="s">
         <v>20</v>
       </c>
@@ -9410,24 +9420,51 @@
       <c r="D11" s="34" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="G11" s="39" t="s">
+        <v>27</v>
+      </c>
+      <c r="H11" s="34" t="s">
+        <v>24</v>
+      </c>
+      <c r="I11" s="34" t="s">
+        <v>25</v>
+      </c>
+      <c r="K11" s="39" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A12" s="35" t="s">
         <v>21</v>
       </c>
       <c r="B12" s="36">
-        <v>3510</v>
+        <v>3514</v>
       </c>
       <c r="C12" s="37">
         <f>VLOOKUP(B12,'Powell-Bathymetry'!$B$2:$C$582,2)/1000000</f>
-        <v>6.433061801</v>
+        <v>6.6449818059999997</v>
       </c>
       <c r="D12" s="37">
         <f>C12-VLOOKUP(3370,'Powell-Bathymetry'!$B$2:$C$582,2)/1000000</f>
-        <v>4.7210644459999997</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+        <v>4.9329844509999994</v>
+      </c>
+      <c r="G12">
+        <v>3545</v>
+      </c>
+      <c r="H12" s="37">
+        <f>VLOOKUP(G12,'Powell-Bathymetry'!$B$2:$C$582,2)/1000000</f>
+        <v>8.4807889360000015</v>
+      </c>
+      <c r="I12" s="37">
+        <f>H12-VLOOKUP(3370,'Powell-Bathymetry'!$B$2:$C$582,2)/1000000</f>
+        <v>6.7687915810000012</v>
+      </c>
+      <c r="K12" s="38">
+        <f>I12-I$16</f>
+        <v>1.8358071300000018</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A13" s="35" t="s">
         <v>22</v>
       </c>
@@ -9441,6 +9478,103 @@
       <c r="D13" s="37">
         <f>VLOOKUP(B$13,'Mead-Bathymetry'!$A$2:$D$673,2)/1000000</f>
         <v>4.475301</v>
+      </c>
+      <c r="G13">
+        <v>3540</v>
+      </c>
+      <c r="H13" s="37">
+        <f>VLOOKUP(G13,'Powell-Bathymetry'!$B$2:$C$582,2)/1000000</f>
+        <v>8.1609592089999996</v>
+      </c>
+      <c r="I13" s="37">
+        <f>H13-VLOOKUP(3370,'Powell-Bathymetry'!$B$2:$C$582,2)/1000000</f>
+        <v>6.4489618539999993</v>
+      </c>
+      <c r="K13" s="38">
+        <f>I13-I$16</f>
+        <v>1.5159774029999999</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="G14">
+        <v>3528</v>
+      </c>
+      <c r="H14" s="37">
+        <f>VLOOKUP(G14,'Powell-Bathymetry'!$B$2:$C$582,2)/1000000</f>
+        <v>7.4311503600000002</v>
+      </c>
+      <c r="I14" s="37">
+        <f>H14-VLOOKUP(3370,'Powell-Bathymetry'!$B$2:$C$582,2)/1000000</f>
+        <v>5.7191530049999999</v>
+      </c>
+      <c r="K14" s="38">
+        <f>I15-I$16</f>
+        <v>0.61193845800000091</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="G15">
+        <v>3525</v>
+      </c>
+      <c r="H15" s="37">
+        <f>VLOOKUP(G15,'Powell-Bathymetry'!$B$2:$C$582,2)/1000000</f>
+        <v>7.2569202640000006</v>
+      </c>
+      <c r="I15" s="37">
+        <f>H15-VLOOKUP(3370,'Powell-Bathymetry'!$B$2:$C$582,2)/1000000</f>
+        <v>5.5449229090000003</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="G16">
+        <v>3514</v>
+      </c>
+      <c r="H16" s="37">
+        <f>VLOOKUP(G16,'Powell-Bathymetry'!$B$2:$C$582,2)/1000000</f>
+        <v>6.6449818059999997</v>
+      </c>
+      <c r="I16" s="37">
+        <f>H16-VLOOKUP(3370,'Powell-Bathymetry'!$B$2:$C$582,2)/1000000</f>
+        <v>4.9329844509999994</v>
+      </c>
+    </row>
+    <row r="17" spans="7:9" x14ac:dyDescent="0.35">
+      <c r="G17">
+        <v>3510</v>
+      </c>
+      <c r="H17" s="37">
+        <f>VLOOKUP(G17,'Powell-Bathymetry'!$B$2:$C$582,2)/1000000</f>
+        <v>6.433061801</v>
+      </c>
+      <c r="I17" s="37">
+        <f>H17-VLOOKUP(3370,'Powell-Bathymetry'!$B$2:$C$582,2)/1000000</f>
+        <v>4.7210644459999997</v>
+      </c>
+    </row>
+    <row r="18" spans="7:9" x14ac:dyDescent="0.35">
+      <c r="G18">
+        <v>3500</v>
+      </c>
+      <c r="H18" s="37">
+        <f>VLOOKUP(G18,'Powell-Bathymetry'!$B$2:$C$582,2)/1000000</f>
+        <v>5.9278024770000002</v>
+      </c>
+      <c r="I18" s="37">
+        <f>H18-VLOOKUP(3370,'Powell-Bathymetry'!$B$2:$C$582,2)/1000000</f>
+        <v>4.2158051219999999</v>
+      </c>
+    </row>
+    <row r="19" spans="7:9" x14ac:dyDescent="0.35">
+      <c r="G19">
+        <v>3490</v>
+      </c>
+      <c r="H19" s="37">
+        <f>VLOOKUP(G19,'Powell-Bathymetry'!$B$2:$C$582,2)/1000000</f>
+        <v>5.4547115049999997</v>
+      </c>
+      <c r="I19" s="37">
+        <f>H19-VLOOKUP(3370,'Powell-Bathymetry'!$B$2:$C$582,2)/1000000</f>
+        <v>3.7427141499999994</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update Elevation Definitions to add Powell 2x Buffer volume
</commit_message>
<xml_diff>
--- a/AutoReadUSBRData/Bathymetry.xlsx
+++ b/AutoReadUSBRData/Bathymetry.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Rosenberg\Work\USU\Research\ColoradoRiver\RCode\ColoradoRiverCollaborate\AutoReadUSBRData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{986D7C98-EC2A-413C-BD64-6CFBD01ADE7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{516BF7B1-2E6E-4F66-A02E-D0567C567724}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-57720" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ReadMe" sheetId="1" r:id="rId1"/>
@@ -428,7 +428,7 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -9360,7 +9360,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K19"/>
+  <dimension ref="A1:L19"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="16.36328125" customWidth="1"/>
@@ -9368,17 +9368,17 @@
     <col min="4" max="4" width="11.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:12" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>12</v>
       </c>
@@ -9386,7 +9386,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>14</v>
       </c>
@@ -9394,7 +9394,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>16</v>
       </c>
@@ -9402,12 +9402,12 @@
         <v>19</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:12" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A11" s="33" t="s">
         <v>20</v>
       </c>
@@ -9433,7 +9433,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A12" s="35" t="s">
         <v>21</v>
       </c>
@@ -9460,11 +9460,11 @@
         <v>6.7687915810000012</v>
       </c>
       <c r="K12" s="38">
-        <f>I12-I$16</f>
+        <f t="shared" ref="K12:K15" si="0">I12-I$16</f>
         <v>1.8358071300000018</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A13" s="35" t="s">
         <v>22</v>
       </c>
@@ -9480,22 +9480,26 @@
         <v>4.475301</v>
       </c>
       <c r="G13">
-        <v>3540</v>
+        <v>3535</v>
       </c>
       <c r="H13" s="37">
         <f>VLOOKUP(G13,'Powell-Bathymetry'!$B$2:$C$582,2)/1000000</f>
-        <v>8.1609592089999996</v>
+        <v>7.8504680980000003</v>
       </c>
       <c r="I13" s="37">
         <f>H13-VLOOKUP(3370,'Powell-Bathymetry'!$B$2:$C$582,2)/1000000</f>
-        <v>6.4489618539999993</v>
+        <v>6.1384707430000001</v>
       </c>
       <c r="K13" s="38">
-        <f>I13-I$16</f>
-        <v>1.5159774029999999</v>
-      </c>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.35">
+        <f t="shared" si="0"/>
+        <v>1.2054862920000007</v>
+      </c>
+      <c r="L13" s="38">
+        <f>I13-I14</f>
+        <v>0.41931773800000016</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.35">
       <c r="G14">
         <v>3528</v>
       </c>
@@ -9508,11 +9512,11 @@
         <v>5.7191530049999999</v>
       </c>
       <c r="K14" s="38">
-        <f>I15-I$16</f>
-        <v>0.61193845800000091</v>
-      </c>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.35">
+        <f t="shared" si="0"/>
+        <v>0.78616855400000052</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.35">
       <c r="G15">
         <v>3525</v>
       </c>
@@ -9524,8 +9528,12 @@
         <f>H15-VLOOKUP(3370,'Powell-Bathymetry'!$B$2:$C$582,2)/1000000</f>
         <v>5.5449229090000003</v>
       </c>
-    </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="K15" s="38">
+        <f t="shared" si="0"/>
+        <v>0.61193845800000091</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.35">
       <c r="G16">
         <v>3514</v>
       </c>
@@ -9536,6 +9544,10 @@
       <c r="I16" s="37">
         <f>H16-VLOOKUP(3370,'Powell-Bathymetry'!$B$2:$C$582,2)/1000000</f>
         <v>4.9329844509999994</v>
+      </c>
+      <c r="K16" s="38">
+        <f>I16-I$16</f>
+        <v>0</v>
       </c>
     </row>
     <row r="17" spans="7:9" x14ac:dyDescent="0.35">

</xml_diff>